<commit_message>
Update hard coal retirement cap to 0.1 based on calibration runs
</commit_message>
<xml_diff>
--- a/InputData/elec/MSoCRiaSY/Maximum Share of Capacity Retired in a Single Year.xlsx
+++ b/InputData/elec/MSoCRiaSY/Maximum Share of Capacity Retired in a Single Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\MSoCRiaSY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9E3443-8B44-4EE4-A2D3-73206D5638AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{833AC9E5-A658-4C59-83BE-7FF35AB20CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4545" yWindow="3765" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -603,7 +603,7 @@
         <v>15</v>
       </c>
       <c r="B2">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Set coal retirement parameter to 0.08
</commit_message>
<xml_diff>
--- a/InputData/elec/MSoCRiaSY/Maximum Share of Capacity Retired in a Single Year.xlsx
+++ b/InputData/elec/MSoCRiaSY/Maximum Share of Capacity Retired in a Single Year.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\MSoCRiaSY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{833AC9E5-A658-4C59-83BE-7FF35AB20CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40ACDC51-D64F-45E5-9022-39C92AFAB2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -603,7 +603,7 @@
         <v>15</v>
       </c>
       <c r="B2">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>